<commit_message>
accounting: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -10782,7 +10782,9 @@
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>Then the home page lists at least the sixteen seeded accounts</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page lists at least the sixteen seeded accounts.</t>
         </is>
       </c>
       <c r="H196" s="3" t="inlineStr">
@@ -10832,7 +10834,9 @@
       </c>
       <c r="G197" s="3" t="inlineStr">
         <is>
-          <t>Then every account row shows a code, a name and a type</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: every account row shows a code, a name and a type.</t>
         </is>
       </c>
       <c r="H197" s="3" t="inlineStr">
@@ -10882,7 +10886,9 @@
       </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
-          <t>Then every account balance on screen is a number</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: every account balance on screen is a number.</t>
         </is>
       </c>
       <c r="H198" s="3" t="inlineStr">
@@ -10932,7 +10938,9 @@
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>Then the home page shows an account of every type</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page shows an account of every type.</t>
         </is>
       </c>
       <c r="H199" s="3" t="inlineStr">
@@ -10982,10 +10990,12 @@
       </c>
       <c r="G200" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a cash sale of 50000
-When the account page for account 1 is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a cash sale of 50000.
+5. Open the app 'Account' screen in the browser (URL /account/1) — on Home, click the row of account 1 in the accounts list.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H200" s="3" t="inlineStr">
@@ -11035,8 +11045,10 @@
       </c>
       <c r="G201" s="3" t="inlineStr">
         <is>
-          <t>When the account page for account 7 is opened
-Then the account page shows code "3000" and type "equity"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Account' screen in the browser (URL /account/7) — on Home, click the row of account 7 in the accounts list.
+4. On screen, verify: the account page shows code "3000" and type "equity".</t>
         </is>
       </c>
       <c r="H201" s="3" t="inlineStr">
@@ -11086,8 +11098,10 @@
       </c>
       <c r="G202" s="3" t="inlineStr">
         <is>
-          <t>When the account page for account 999999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Account' screen in the browser (URL /account/999999) — on Home, click the row of account 999999 in the accounts list.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H202" s="3" t="inlineStr">
@@ -11137,10 +11151,12 @@
       </c>
       <c r="G203" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a cash sale of 30000
-When the entry page is opened
-Then the entry lines on screen show a debit and a credit of the same amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a cash sale of 30000.
+5. Open the app 'Journal Entry' screen in the browser (URL /entry/&lt;the entry just posted&gt;) — click the just-posted entry's link.
+6. On screen, verify: the entry lines on screen show a debit and a credit of the same amount.</t>
         </is>
       </c>
       <c r="H203" s="3" t="inlineStr">
@@ -11190,10 +11206,12 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a cash sale of 30000
-When the entry page is opened
-Then the entry page shows status "posted"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a cash sale of 30000.
+5. Open the app 'Journal Entry' screen in the browser (URL /entry/&lt;the entry just posted&gt;) — click the just-posted entry's link.
+6. On screen, verify: the entry page shows status "posted".</t>
         </is>
       </c>
       <c r="H204" s="3" t="inlineStr">
@@ -11243,11 +11261,13 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a cash sale of 30000
-And the entry is reversed by the admin
-When the entry page is opened
-Then the entry page shows status "reversed"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a cash sale of 30000.
+5. Set up (before checking the screen): the entry is reversed by the admin.
+6. Open the app 'Journal Entry' screen in the browser (URL /entry/&lt;the entry just posted&gt;) — click the just-posted entry's link.
+7. On screen, verify: the entry page shows status "reversed".</t>
         </is>
       </c>
       <c r="H205" s="3" t="inlineStr">
@@ -11297,8 +11317,10 @@
       </c>
       <c r="G206" s="3" t="inlineStr">
         <is>
-          <t>When the entry page for 999999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Journal Entry' screen in the browser (URL /entry/999999) — click the link for entry 999999.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H206" s="3" t="inlineStr">
@@ -11348,9 +11370,11 @@
       </c>
       <c r="G207" s="3" t="inlineStr">
         <is>
-          <t>When the trial balance page is opened
-Then the trial balance page shows the debits equal the credits
-And the trial balance page shows it balanced</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Trial Balance report' screen in the browser (URL /trial-balance) — on Home, click 'Trial Balance'.
+4. On screen, verify: the trial balance page shows the debits equal the credits.
+5. On screen, verify: the trial balance page shows it balanced.</t>
         </is>
       </c>
       <c r="H207" s="3" t="inlineStr">
@@ -11401,10 +11425,12 @@
       </c>
       <c r="G208" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a cash sale of 45000
-When the trial balance page is opened
-Then the trial balance page shows it balanced</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a cash sale of 45000.
+5. Open the app 'Trial Balance report' screen in the browser (URL /trial-balance) — on Home, click 'Trial Balance'.
+6. On screen, verify: the trial balance page shows it balanced.</t>
         </is>
       </c>
       <c r="H208" s="3" t="inlineStr">
@@ -11454,9 +11480,11 @@
       </c>
       <c r="G209" s="3" t="inlineStr">
         <is>
-          <t>When the balance sheet page is opened
-Then the balance sheet page shows Assets equal Liabilities plus Equity plus Net income
-And the balance sheet page shows it balanced</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Balance Sheet report' screen in the browser (URL /balance-sheet) — on Home, click 'Balance Sheet'.
+4. On screen, verify: the balance sheet page shows Assets equal Liabilities plus Equity plus Net income.
+5. On screen, verify: the balance sheet page shows it balanced.</t>
         </is>
       </c>
       <c r="H209" s="3" t="inlineStr">
@@ -11507,10 +11535,12 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account 4 and crediting account 5 for 250000
-When the balance sheet page is opened
-Then the balance sheet page shows it balanced</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account 4 and crediting account 5 for 250000.
+5. Open the app 'Balance Sheet report' screen in the browser (URL /balance-sheet) — on Home, click 'Balance Sheet'.
+6. On screen, verify: the balance sheet page shows it balanced.</t>
         </is>
       </c>
       <c r="H210" s="3" t="inlineStr">
@@ -11560,8 +11590,10 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then the admin page shows it balanced</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: the admin page shows it balanced.</t>
         </is>
       </c>
       <c r="H211" s="3" t="inlineStr">
@@ -11611,8 +11643,10 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then the admin entry count is a positive integer</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: the admin entry count is a positive integer.</t>
         </is>
       </c>
       <c r="H212" s="3" t="inlineStr">
@@ -11662,10 +11696,12 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H213" s="3" t="inlineStr">
@@ -11715,10 +11751,12 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H214" s="3" t="inlineStr">
@@ -11768,10 +11806,12 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H215" s="3" t="inlineStr">
@@ -11821,10 +11861,12 @@
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 9 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H216" s="3" t="inlineStr">
@@ -23747,10 +23789,12 @@
       </c>
       <c r="G441" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H441" s="3" t="inlineStr">
@@ -23800,10 +23844,12 @@
       </c>
       <c r="G442" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H442" s="3" t="inlineStr">
@@ -23853,10 +23899,12 @@
       </c>
       <c r="G443" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H443" s="3" t="inlineStr">
@@ -23906,10 +23954,12 @@
       </c>
       <c r="G444" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H444" s="3" t="inlineStr">
@@ -23959,10 +24009,12 @@
       </c>
       <c r="G445" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H445" s="3" t="inlineStr">
@@ -24012,10 +24064,12 @@
       </c>
       <c r="G446" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H446" s="3" t="inlineStr">
@@ -24065,10 +24119,12 @@
       </c>
       <c r="G447" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H447" s="3" t="inlineStr">
@@ -24118,10 +24174,12 @@
       </c>
       <c r="G448" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H448" s="3" t="inlineStr">
@@ -24171,10 +24229,12 @@
       </c>
       <c r="G449" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H449" s="3" t="inlineStr">
@@ -24224,10 +24284,12 @@
       </c>
       <c r="G450" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H450" s="3" t="inlineStr">
@@ -24277,10 +24339,12 @@
       </c>
       <c r="G451" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H451" s="3" t="inlineStr">
@@ -24330,10 +24394,12 @@
       </c>
       <c r="G452" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H452" s="3" t="inlineStr">
@@ -24383,10 +24449,12 @@
       </c>
       <c r="G453" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H453" s="3" t="inlineStr">
@@ -24436,10 +24504,12 @@
       </c>
       <c r="G454" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H454" s="3" t="inlineStr">
@@ -24489,10 +24559,12 @@
       </c>
       <c r="G455" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H455" s="3" t="inlineStr">
@@ -24542,10 +24614,12 @@
       </c>
       <c r="G456" s="3" t="inlineStr">
         <is>
-          <t>Given an accountant
-And a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;
-When the account page for account &lt;acc&gt; is opened
-Then the account page balance equals the stored balance</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – chart of accounts' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): an accountant.
+4. Set up (before checking the screen): a balanced entry debiting account &lt;acc&gt; and crediting account 10 for &lt;amount&gt;.
+5. Set up (before checking the screen): the account page for account &lt;acc&gt; is opened.
+6. On screen, verify: the account page balance equals the stored balance.</t>
         </is>
       </c>
       <c r="H456" s="3" t="inlineStr">

</xml_diff>